<commit_message>
fix(web-padre): update version timestamp to trigger vercel build
</commit_message>
<xml_diff>
--- a/clientes/prospectos_caba.xlsx
+++ b/clientes/prospectos_caba.xlsx
@@ -490,7 +490,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L47"/>
+  <dimension ref="A1:L106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -499,7 +499,7 @@
     <col width="21" customWidth="1" min="4" max="4"/>
     <col width="48" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="36" customWidth="1" min="7" max="7"/>
+    <col width="43" customWidth="1" min="7" max="7"/>
     <col width="29" customWidth="1" min="8" max="8"/>
     <col width="29" customWidth="1" min="9" max="9"/>
     <col width="22" customWidth="1" min="10" max="10"/>
@@ -3232,6 +3232,3428 @@
       </c>
       <c r="K47" s="2" t="inlineStr"/>
       <c r="L47" s="7" t="inlineStr">
+        <is>
+          <t>Ver en Maps</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="22" customHeight="1">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>PELUQUERÍA Y PETSHOP FULLMASKOTAS</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>PELUQUERÍA Y PETSHOP FULLMASKOTAS</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>Mascotas / Pet Shop</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>011 15-7656-6041</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>Malabia 2284, C1425 Cdad. Autónoma de Buenos Aires</t>
+        </is>
+      </c>
+      <c r="F48" s="3" t="inlineStr">
+        <is>
+          <t>4.5</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>E-commerce WhatsApp &amp; Turnos Peluquería</t>
+        </is>
+      </c>
+      <c r="H48" s="4" t="inlineStr">
+        <is>
+          <t>📲 Enviar Mensaje</t>
+        </is>
+      </c>
+      <c r="I48" s="5" t="inlineStr">
+        <is>
+          <t>🔗 Probar Boceto</t>
+        </is>
+      </c>
+      <c r="J48" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="K48" s="2" t="inlineStr"/>
+      <c r="L48" s="7" t="inlineStr">
+        <is>
+          <t>Ver en Maps</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="22" customHeight="1">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>Petba Pet Shop - Veterinaria - Peluquería Canina - Av. Belgrano 1737</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>Petba Pet Shop - Veterinaria - Peluquería Canina - Av. Belgrano 1737</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>Mascotas / Pet Shop</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>011 4381-0359</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>Av. Belgrano 1737, C1093AAF Cdad. Autónoma de Buenos Aires</t>
+        </is>
+      </c>
+      <c r="F49" s="3" t="inlineStr">
+        <is>
+          <t>4.1</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
+          <t>E-commerce WhatsApp &amp; Turnos Peluquería</t>
+        </is>
+      </c>
+      <c r="H49" s="4" t="inlineStr">
+        <is>
+          <t>📲 Enviar Mensaje</t>
+        </is>
+      </c>
+      <c r="I49" s="5" t="inlineStr">
+        <is>
+          <t>🔗 Probar Boceto</t>
+        </is>
+      </c>
+      <c r="J49" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="K49" s="2" t="inlineStr"/>
+      <c r="L49" s="7" t="inlineStr">
+        <is>
+          <t>Ver en Maps</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="22" customHeight="1">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>Petba Pet Shop &amp; Peluquería - Av. Entre Ríos 233 - NOS MUDAMOS A AV. BELGRANO 1737</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>Petba Pet Shop &amp; Peluquería - Av. Entre Ríos 233 - NOS MUDAMOS A AV. BELGRANO 1737</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>Mascotas / Pet Shop</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>011 4381-0359</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>Av. Entre Ríos 233, C1079ABC Cdad. Autónoma de Buenos Aires</t>
+        </is>
+      </c>
+      <c r="F50" s="3" t="inlineStr">
+        <is>
+          <t>3.9</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>E-commerce WhatsApp &amp; Turnos Peluquería</t>
+        </is>
+      </c>
+      <c r="H50" s="4" t="inlineStr">
+        <is>
+          <t>📲 Enviar Mensaje</t>
+        </is>
+      </c>
+      <c r="I50" s="5" t="inlineStr">
+        <is>
+          <t>🔗 Probar Boceto</t>
+        </is>
+      </c>
+      <c r="J50" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="K50" s="2" t="inlineStr"/>
+      <c r="L50" s="7" t="inlineStr">
+        <is>
+          <t>Ver en Maps</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="22" customHeight="1">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>Bírichini pet</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>Bírichini pet</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>Mascotas / Pet Shop</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>011 4901-0380</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>Rosario 751 C1424CCO, C1424CCO Cdad. Autónoma de Buenos Aires</t>
+        </is>
+      </c>
+      <c r="F51" s="3" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="inlineStr">
+        <is>
+          <t>E-commerce WhatsApp &amp; Turnos Peluquería</t>
+        </is>
+      </c>
+      <c r="H51" s="4" t="inlineStr">
+        <is>
+          <t>📲 Enviar Mensaje</t>
+        </is>
+      </c>
+      <c r="I51" s="5" t="inlineStr">
+        <is>
+          <t>🔗 Probar Boceto</t>
+        </is>
+      </c>
+      <c r="J51" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="K51" s="2" t="inlineStr"/>
+      <c r="L51" s="7" t="inlineStr">
+        <is>
+          <t>Ver en Maps</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="22" customHeight="1">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>Pet Shop Caninos</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>Pet Shop Caninos</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>Mascotas / Pet Shop</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>011 6496-7250</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>Av. Juan Bautista Alberdi 931, C1424BYJ Cdad. Autónoma de Buenos Aires</t>
+        </is>
+      </c>
+      <c r="F52" s="3" t="inlineStr">
+        <is>
+          <t>4.3</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t>E-commerce WhatsApp &amp; Turnos Peluquería</t>
+        </is>
+      </c>
+      <c r="H52" s="4" t="inlineStr">
+        <is>
+          <t>📲 Enviar Mensaje</t>
+        </is>
+      </c>
+      <c r="I52" s="5" t="inlineStr">
+        <is>
+          <t>🔗 Probar Boceto</t>
+        </is>
+      </c>
+      <c r="J52" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="K52" s="2" t="inlineStr"/>
+      <c r="L52" s="7" t="inlineStr">
+        <is>
+          <t>Ver en Maps</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="22" customHeight="1">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>Huesitos Pet shop</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>Huesitos Pet shop</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>Mascotas / Pet Shop</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>011 4319-7506</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>Yerbal 887, C1405 C1405CDQ, Cdad. Autónoma de Buenos Aires</t>
+        </is>
+      </c>
+      <c r="F53" s="3" t="inlineStr">
+        <is>
+          <t>4.8</t>
+        </is>
+      </c>
+      <c r="G53" s="2" t="inlineStr">
+        <is>
+          <t>E-commerce WhatsApp &amp; Turnos Peluquería</t>
+        </is>
+      </c>
+      <c r="H53" s="4" t="inlineStr">
+        <is>
+          <t>📲 Enviar Mensaje</t>
+        </is>
+      </c>
+      <c r="I53" s="5" t="inlineStr">
+        <is>
+          <t>🔗 Probar Boceto</t>
+        </is>
+      </c>
+      <c r="J53" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="K53" s="2" t="inlineStr"/>
+      <c r="L53" s="7" t="inlineStr">
+        <is>
+          <t>Ver en Maps</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="22" customHeight="1">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>AREA PET</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>AREA PET</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>Mascotas / Pet Shop</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>011 4853-2549</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>Juncal 2731, C1425AYG Cdad. Autónoma de Buenos Aires</t>
+        </is>
+      </c>
+      <c r="F54" s="3" t="inlineStr">
+        <is>
+          <t>4.5</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t>E-commerce WhatsApp &amp; Turnos Peluquería</t>
+        </is>
+      </c>
+      <c r="H54" s="4" t="inlineStr">
+        <is>
+          <t>📲 Enviar Mensaje</t>
+        </is>
+      </c>
+      <c r="I54" s="5" t="inlineStr">
+        <is>
+          <t>🔗 Probar Boceto</t>
+        </is>
+      </c>
+      <c r="J54" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="K54" s="2" t="inlineStr"/>
+      <c r="L54" s="7" t="inlineStr">
+        <is>
+          <t>Ver en Maps</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="22" customHeight="1">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>King &amp; Queen Pet Shop</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>King &amp; Queen Pet Shop</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>Mascotas / Pet Shop</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>011 15-2165-6136</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>Sánchez de Bustamante 1661, C1425DUG Cdad. Autónoma de Buenos Aires</t>
+        </is>
+      </c>
+      <c r="F55" s="3" t="inlineStr">
+        <is>
+          <t>4.6</t>
+        </is>
+      </c>
+      <c r="G55" s="2" t="inlineStr">
+        <is>
+          <t>E-commerce WhatsApp &amp; Turnos Peluquería</t>
+        </is>
+      </c>
+      <c r="H55" s="4" t="inlineStr">
+        <is>
+          <t>📲 Enviar Mensaje</t>
+        </is>
+      </c>
+      <c r="I55" s="5" t="inlineStr">
+        <is>
+          <t>🔗 Probar Boceto</t>
+        </is>
+      </c>
+      <c r="J55" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="K55" s="2" t="inlineStr"/>
+      <c r="L55" s="7" t="inlineStr">
+        <is>
+          <t>Ver en Maps</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="22" customHeight="1">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>Kiki Pet Shop &amp; Bath</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>Kiki Pet Shop &amp; Bath</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>Mascotas / Pet Shop</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>011 15-4029-6216</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>Laprida 1290, C1425 Cdad. Autónoma de Buenos Aires</t>
+        </is>
+      </c>
+      <c r="F56" s="3" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="inlineStr">
+        <is>
+          <t>E-commerce WhatsApp &amp; Turnos Peluquería</t>
+        </is>
+      </c>
+      <c r="H56" s="4" t="inlineStr">
+        <is>
+          <t>📲 Enviar Mensaje</t>
+        </is>
+      </c>
+      <c r="I56" s="5" t="inlineStr">
+        <is>
+          <t>🔗 Probar Boceto</t>
+        </is>
+      </c>
+      <c r="J56" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="K56" s="2" t="inlineStr"/>
+      <c r="L56" s="7" t="inlineStr">
+        <is>
+          <t>Ver en Maps</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="22" customHeight="1">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>Petshop Leo y Axel</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>Petshop Leo y Axel</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>Mascotas / Pet Shop</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>011 7358-3408</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>Juan Ramírez de Velasco 175, C1414 Cdad. Autónoma de Buenos Aires</t>
+        </is>
+      </c>
+      <c r="F57" s="3" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="G57" s="2" t="inlineStr">
+        <is>
+          <t>E-commerce WhatsApp &amp; Turnos Peluquería</t>
+        </is>
+      </c>
+      <c r="H57" s="4" t="inlineStr">
+        <is>
+          <t>📲 Enviar Mensaje</t>
+        </is>
+      </c>
+      <c r="I57" s="5" t="inlineStr">
+        <is>
+          <t>🔗 Probar Boceto</t>
+        </is>
+      </c>
+      <c r="J57" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="K57" s="2" t="inlineStr"/>
+      <c r="L57" s="7" t="inlineStr">
+        <is>
+          <t>Ver en Maps</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="22" customHeight="1">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>Pet Friendly</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>Pet Friendly</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>Mascotas / Pet Shop</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>011 2359-9913</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>Vera 21, C1414AOA Cdad. Autónoma de Buenos Aires</t>
+        </is>
+      </c>
+      <c r="F58" s="3" t="inlineStr">
+        <is>
+          <t>4.9</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t>E-commerce WhatsApp &amp; Turnos Peluquería</t>
+        </is>
+      </c>
+      <c r="H58" s="4" t="inlineStr">
+        <is>
+          <t>📲 Enviar Mensaje</t>
+        </is>
+      </c>
+      <c r="I58" s="5" t="inlineStr">
+        <is>
+          <t>🔗 Probar Boceto</t>
+        </is>
+      </c>
+      <c r="J58" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="K58" s="2" t="inlineStr"/>
+      <c r="L58" s="7" t="inlineStr">
+        <is>
+          <t>Ver en Maps</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="22" customHeight="1">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>DISTRICAN</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>DISTRICAN</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>Mascotas / Pet Shop</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>011 4857-1441</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="inlineStr">
+        <is>
+          <t>Av. Warnes 342, C1414 AAQ, Cdad. Autónoma de Buenos Aires</t>
+        </is>
+      </c>
+      <c r="F59" s="3" t="inlineStr">
+        <is>
+          <t>4.8</t>
+        </is>
+      </c>
+      <c r="G59" s="2" t="inlineStr">
+        <is>
+          <t>E-commerce WhatsApp &amp; Turnos Peluquería</t>
+        </is>
+      </c>
+      <c r="H59" s="4" t="inlineStr">
+        <is>
+          <t>📲 Enviar Mensaje</t>
+        </is>
+      </c>
+      <c r="I59" s="5" t="inlineStr">
+        <is>
+          <t>🔗 Probar Boceto</t>
+        </is>
+      </c>
+      <c r="J59" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="K59" s="2" t="inlineStr"/>
+      <c r="L59" s="7" t="inlineStr">
+        <is>
+          <t>Ver en Maps</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="22" customHeight="1">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>Pet Shop Grandes Amigos</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>Pet Shop Grandes Amigos</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>Mascotas / Pet Shop</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>011 3119-1969</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>Quintino Bocayuva 224, C1181 AAF, Cdad. Autónoma de Buenos Aires</t>
+        </is>
+      </c>
+      <c r="F60" s="3" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="G60" s="2" t="inlineStr">
+        <is>
+          <t>E-commerce WhatsApp &amp; Turnos Peluquería</t>
+        </is>
+      </c>
+      <c r="H60" s="4" t="inlineStr">
+        <is>
+          <t>📲 Enviar Mensaje</t>
+        </is>
+      </c>
+      <c r="I60" s="5" t="inlineStr">
+        <is>
+          <t>🔗 Probar Boceto</t>
+        </is>
+      </c>
+      <c r="J60" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="K60" s="2" t="inlineStr"/>
+      <c r="L60" s="7" t="inlineStr">
+        <is>
+          <t>Ver en Maps</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="22" customHeight="1">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>Don Simon Pet Shop</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>Don Simon Pet Shop</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>Mascotas / Pet Shop</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>011 6139-3016</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="inlineStr">
+        <is>
+          <t>Castro Barros 787, C1217 Cdad. Autónoma de Buenos Aires</t>
+        </is>
+      </c>
+      <c r="F61" s="3" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="G61" s="2" t="inlineStr">
+        <is>
+          <t>E-commerce WhatsApp &amp; Turnos Peluquería</t>
+        </is>
+      </c>
+      <c r="H61" s="4" t="inlineStr">
+        <is>
+          <t>📲 Enviar Mensaje</t>
+        </is>
+      </c>
+      <c r="I61" s="5" t="inlineStr">
+        <is>
+          <t>🔗 Probar Boceto</t>
+        </is>
+      </c>
+      <c r="J61" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="K61" s="2" t="inlineStr"/>
+      <c r="L61" s="7" t="inlineStr">
+        <is>
+          <t>Ver en Maps</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="22" customHeight="1">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>Pet Shop León Urquiza</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>Pet Shop León Urquiza</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>Mascotas / Pet Shop</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>011 15-6980-1155</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>Blanco Encalada 5075, Villa Urquiza, Juramento 5032, C1431 Cdad. Autónoma de Buenos Aires</t>
+        </is>
+      </c>
+      <c r="F62" s="3" t="inlineStr">
+        <is>
+          <t>4.4</t>
+        </is>
+      </c>
+      <c r="G62" s="2" t="inlineStr">
+        <is>
+          <t>E-commerce WhatsApp &amp; Turnos Peluquería</t>
+        </is>
+      </c>
+      <c r="H62" s="4" t="inlineStr">
+        <is>
+          <t>📲 Enviar Mensaje</t>
+        </is>
+      </c>
+      <c r="I62" s="5" t="inlineStr">
+        <is>
+          <t>🔗 Probar Boceto</t>
+        </is>
+      </c>
+      <c r="J62" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="K62" s="2" t="inlineStr"/>
+      <c r="L62" s="7" t="inlineStr">
+        <is>
+          <t>Ver en Maps</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="22" customHeight="1">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>FOR PET VETERINARIA</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>FOR PET VETERINARIA</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>Mascotas / Pet Shop</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>011 4523-2216</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="inlineStr">
+        <is>
+          <t>Altolaguirre 1803, C1431ECI Cdad. Autónoma de Buenos Aires</t>
+        </is>
+      </c>
+      <c r="F63" s="3" t="inlineStr">
+        <is>
+          <t>4.6</t>
+        </is>
+      </c>
+      <c r="G63" s="2" t="inlineStr">
+        <is>
+          <t>E-commerce WhatsApp &amp; Turnos Peluquería</t>
+        </is>
+      </c>
+      <c r="H63" s="4" t="inlineStr">
+        <is>
+          <t>📲 Enviar Mensaje</t>
+        </is>
+      </c>
+      <c r="I63" s="5" t="inlineStr">
+        <is>
+          <t>🔗 Probar Boceto</t>
+        </is>
+      </c>
+      <c r="J63" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="K63" s="2" t="inlineStr"/>
+      <c r="L63" s="7" t="inlineStr">
+        <is>
+          <t>Ver en Maps</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="22" customHeight="1">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>Veterinaria y Pet Shop PuntoVet Villa Urquiza</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>Veterinaria y Pet Shop PuntoVet Villa Urquiza</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>Mascotas / Pet Shop</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>011 3183-5444</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="inlineStr">
+        <is>
+          <t>Av. Olazábal 5601, C1431 Cdad. Autónoma de Buenos Aires</t>
+        </is>
+      </c>
+      <c r="F64" s="3" t="inlineStr">
+        <is>
+          <t>4.6</t>
+        </is>
+      </c>
+      <c r="G64" s="2" t="inlineStr">
+        <is>
+          <t>E-commerce WhatsApp &amp; Turnos Peluquería</t>
+        </is>
+      </c>
+      <c r="H64" s="4" t="inlineStr">
+        <is>
+          <t>📲 Enviar Mensaje</t>
+        </is>
+      </c>
+      <c r="I64" s="5" t="inlineStr">
+        <is>
+          <t>🔗 Probar Boceto</t>
+        </is>
+      </c>
+      <c r="J64" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="K64" s="2" t="inlineStr"/>
+      <c r="L64" s="7" t="inlineStr">
+        <is>
+          <t>Ver en Maps</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="22" customHeight="1">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>Estación Mascotas</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>Estación Mascotas</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>Mascotas / Pet Shop</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>011 2462-0653</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="inlineStr">
+        <is>
+          <t>Blanco Encalada 4760, C1431CDH Cdad. Autónoma de Buenos Aires</t>
+        </is>
+      </c>
+      <c r="F65" s="3" t="inlineStr">
+        <is>
+          <t>4.8</t>
+        </is>
+      </c>
+      <c r="G65" s="2" t="inlineStr">
+        <is>
+          <t>E-commerce WhatsApp &amp; Turnos Peluquería</t>
+        </is>
+      </c>
+      <c r="H65" s="4" t="inlineStr">
+        <is>
+          <t>📲 Enviar Mensaje</t>
+        </is>
+      </c>
+      <c r="I65" s="5" t="inlineStr">
+        <is>
+          <t>🔗 Probar Boceto</t>
+        </is>
+      </c>
+      <c r="J65" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="K65" s="2" t="inlineStr"/>
+      <c r="L65" s="7" t="inlineStr">
+        <is>
+          <t>Ver en Maps</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="22" customHeight="1">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>petshop leon</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>Petshop Leon</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>Mascotas / Pet Shop</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>011 6825-7391</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t>Av. Triunvirato 4842, C1431 Cdad. Autónoma de Buenos Aires</t>
+        </is>
+      </c>
+      <c r="F66" s="3" t="inlineStr">
+        <is>
+          <t>4.9</t>
+        </is>
+      </c>
+      <c r="G66" s="2" t="inlineStr">
+        <is>
+          <t>E-commerce WhatsApp &amp; Turnos Peluquería</t>
+        </is>
+      </c>
+      <c r="H66" s="4" t="inlineStr">
+        <is>
+          <t>📲 Enviar Mensaje</t>
+        </is>
+      </c>
+      <c r="I66" s="5" t="inlineStr">
+        <is>
+          <t>🔗 Probar Boceto</t>
+        </is>
+      </c>
+      <c r="J66" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="K66" s="2" t="inlineStr"/>
+      <c r="L66" s="7" t="inlineStr">
+        <is>
+          <t>Ver en Maps</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="22" customHeight="1">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>Tinto Pet Louis</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>Tinto Pet Louis</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>Mascotas / Pet Shop</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr">
+        <is>
+          <t>011 2766-3489</t>
+        </is>
+      </c>
+      <c r="E67" s="2" t="inlineStr">
+        <is>
+          <t>Bucarelli 2592, C1431DRD Cdad. Autónoma de Buenos Aires</t>
+        </is>
+      </c>
+      <c r="F67" s="3" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="G67" s="2" t="inlineStr">
+        <is>
+          <t>E-commerce WhatsApp &amp; Turnos Peluquería</t>
+        </is>
+      </c>
+      <c r="H67" s="4" t="inlineStr">
+        <is>
+          <t>📲 Enviar Mensaje</t>
+        </is>
+      </c>
+      <c r="I67" s="5" t="inlineStr">
+        <is>
+          <t>🔗 Probar Boceto</t>
+        </is>
+      </c>
+      <c r="J67" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="K67" s="2" t="inlineStr"/>
+      <c r="L67" s="7" t="inlineStr">
+        <is>
+          <t>Ver en Maps</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="22" customHeight="1">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>Tinto Pet</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>Tinto Pet</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>Mascotas / Pet Shop</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>011 2382-9939</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="inlineStr">
+        <is>
+          <t>Mariano Acha 2719, C1430 Cdad. Autónoma de Buenos Aires</t>
+        </is>
+      </c>
+      <c r="F68" s="3" t="inlineStr">
+        <is>
+          <t>4.6</t>
+        </is>
+      </c>
+      <c r="G68" s="2" t="inlineStr">
+        <is>
+          <t>E-commerce WhatsApp &amp; Turnos Peluquería</t>
+        </is>
+      </c>
+      <c r="H68" s="4" t="inlineStr">
+        <is>
+          <t>📲 Enviar Mensaje</t>
+        </is>
+      </c>
+      <c r="I68" s="5" t="inlineStr">
+        <is>
+          <t>🔗 Probar Boceto</t>
+        </is>
+      </c>
+      <c r="J68" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="K68" s="2" t="inlineStr"/>
+      <c r="L68" s="7" t="inlineStr">
+        <is>
+          <t>Ver en Maps</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="22" customHeight="1">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>Animal Beauty</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>Animal Beauty</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>Mascotas / Pet Shop</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="inlineStr">
+        <is>
+          <t>011 7525-5634</t>
+        </is>
+      </c>
+      <c r="E69" s="2" t="inlineStr">
+        <is>
+          <t>Quesada 4500, C1430AYH Cdad. Autónoma de Buenos Aires</t>
+        </is>
+      </c>
+      <c r="F69" s="3" t="inlineStr">
+        <is>
+          <t>4.7</t>
+        </is>
+      </c>
+      <c r="G69" s="2" t="inlineStr">
+        <is>
+          <t>E-commerce WhatsApp &amp; Turnos Peluquería</t>
+        </is>
+      </c>
+      <c r="H69" s="4" t="inlineStr">
+        <is>
+          <t>📲 Enviar Mensaje</t>
+        </is>
+      </c>
+      <c r="I69" s="5" t="inlineStr">
+        <is>
+          <t>🔗 Probar Boceto</t>
+        </is>
+      </c>
+      <c r="J69" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="K69" s="2" t="inlineStr"/>
+      <c r="L69" s="7" t="inlineStr">
+        <is>
+          <t>Ver en Maps</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="22" customHeight="1">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>Planeta Mascota Flores</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>Planeta Mascota Flores</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>Mascotas / Pet Shop</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>011 15-5334-4473</t>
+        </is>
+      </c>
+      <c r="E70" s="2" t="inlineStr">
+        <is>
+          <t>Cnel. Ramón L. Falcón 2212, C1406 Cdad. Autónoma de Buenos Aires</t>
+        </is>
+      </c>
+      <c r="F70" s="3" t="inlineStr">
+        <is>
+          <t>4.8</t>
+        </is>
+      </c>
+      <c r="G70" s="2" t="inlineStr">
+        <is>
+          <t>E-commerce WhatsApp &amp; Turnos Peluquería</t>
+        </is>
+      </c>
+      <c r="H70" s="4" t="inlineStr">
+        <is>
+          <t>📲 Enviar Mensaje</t>
+        </is>
+      </c>
+      <c r="I70" s="5" t="inlineStr">
+        <is>
+          <t>🔗 Probar Boceto</t>
+        </is>
+      </c>
+      <c r="J70" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="K70" s="2" t="inlineStr"/>
+      <c r="L70" s="7" t="inlineStr">
+        <is>
+          <t>Ver en Maps</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="22" customHeight="1">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>Pet Shop El bulldog - Huellitas</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>Pet Shop El bulldog - Huellitas</t>
+        </is>
+      </c>
+      <c r="C71" s="2" t="inlineStr">
+        <is>
+          <t>Mascotas / Pet Shop</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="inlineStr">
+        <is>
+          <t>011 6977-0605</t>
+        </is>
+      </c>
+      <c r="E71" s="2" t="inlineStr">
+        <is>
+          <t>Av. Directorio 1508, C1406 Buenos Aires, C.f.</t>
+        </is>
+      </c>
+      <c r="F71" s="3" t="inlineStr">
+        <is>
+          <t>4.7</t>
+        </is>
+      </c>
+      <c r="G71" s="2" t="inlineStr">
+        <is>
+          <t>E-commerce WhatsApp &amp; Turnos Peluquería</t>
+        </is>
+      </c>
+      <c r="H71" s="4" t="inlineStr">
+        <is>
+          <t>📲 Enviar Mensaje</t>
+        </is>
+      </c>
+      <c r="I71" s="5" t="inlineStr">
+        <is>
+          <t>🔗 Probar Boceto</t>
+        </is>
+      </c>
+      <c r="J71" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="K71" s="2" t="inlineStr"/>
+      <c r="L71" s="7" t="inlineStr">
+        <is>
+          <t>Ver en Maps</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="22" customHeight="1">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>La Porteña Pet Shop &amp; Gardening</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>La Porteña Pet Shop &amp; Gardening</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>Mascotas / Pet Shop</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>2055-9104</t>
+        </is>
+      </c>
+      <c r="E72" s="2" t="inlineStr">
+        <is>
+          <t>Av. Juan Bautista Alberdi 927, C1424BYJ Cdad. Autónoma de Buenos Aires</t>
+        </is>
+      </c>
+      <c r="F72" s="3" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="G72" s="2" t="inlineStr">
+        <is>
+          <t>E-commerce WhatsApp &amp; Turnos Peluquería</t>
+        </is>
+      </c>
+      <c r="H72" s="4" t="inlineStr">
+        <is>
+          <t>📲 Enviar Mensaje</t>
+        </is>
+      </c>
+      <c r="I72" s="5" t="inlineStr">
+        <is>
+          <t>🔗 Probar Boceto</t>
+        </is>
+      </c>
+      <c r="J72" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="K72" s="2" t="inlineStr"/>
+      <c r="L72" s="7" t="inlineStr">
+        <is>
+          <t>Ver en Maps</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="22" customHeight="1">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>Pet Shop Multimascota Flores</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>Pet Shop Multimascota Flores</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="inlineStr">
+        <is>
+          <t>Mascotas / Pet Shop</t>
+        </is>
+      </c>
+      <c r="D73" s="2" t="inlineStr">
+        <is>
+          <t>011 2326-0222</t>
+        </is>
+      </c>
+      <c r="E73" s="2" t="inlineStr">
+        <is>
+          <t>Camacuá 27, C1406DOA Cdad. Autónoma de Buenos Aires</t>
+        </is>
+      </c>
+      <c r="F73" s="3" t="inlineStr">
+        <is>
+          <t>4.5</t>
+        </is>
+      </c>
+      <c r="G73" s="2" t="inlineStr">
+        <is>
+          <t>E-commerce WhatsApp &amp; Turnos Peluquería</t>
+        </is>
+      </c>
+      <c r="H73" s="4" t="inlineStr">
+        <is>
+          <t>📲 Enviar Mensaje</t>
+        </is>
+      </c>
+      <c r="I73" s="5" t="inlineStr">
+        <is>
+          <t>🔗 Probar Boceto</t>
+        </is>
+      </c>
+      <c r="J73" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="K73" s="2" t="inlineStr"/>
+      <c r="L73" s="7" t="inlineStr">
+        <is>
+          <t>Ver en Maps</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="22" customHeight="1">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>PET SHOP Del Parque</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>PET SHOP Del Parque</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>Mascotas / Pet Shop</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="inlineStr">
+        <is>
+          <t>011 3793-7921</t>
+        </is>
+      </c>
+      <c r="E74" s="2" t="inlineStr">
+        <is>
+          <t>Av. Eva Perón 1571, C1406 Cdad. Autónoma de Buenos Aires</t>
+        </is>
+      </c>
+      <c r="F74" s="3" t="inlineStr">
+        <is>
+          <t>4.6</t>
+        </is>
+      </c>
+      <c r="G74" s="2" t="inlineStr">
+        <is>
+          <t>E-commerce WhatsApp &amp; Turnos Peluquería</t>
+        </is>
+      </c>
+      <c r="H74" s="4" t="inlineStr">
+        <is>
+          <t>📲 Enviar Mensaje</t>
+        </is>
+      </c>
+      <c r="I74" s="5" t="inlineStr">
+        <is>
+          <t>🔗 Probar Boceto</t>
+        </is>
+      </c>
+      <c r="J74" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="K74" s="2" t="inlineStr"/>
+      <c r="L74" s="7" t="inlineStr">
+        <is>
+          <t>Ver en Maps</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="22" customHeight="1">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>Lucky PET SHOP</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>Lucky PET SHOP</t>
+        </is>
+      </c>
+      <c r="C75" s="2" t="inlineStr">
+        <is>
+          <t>Mascotas / Pet Shop</t>
+        </is>
+      </c>
+      <c r="D75" s="2" t="inlineStr">
+        <is>
+          <t>011 3434-8141</t>
+        </is>
+      </c>
+      <c r="E75" s="2" t="inlineStr">
+        <is>
+          <t>Sanabria 2750, C1417 Cdad. Autónoma de Buenos Aires</t>
+        </is>
+      </c>
+      <c r="F75" s="3" t="inlineStr">
+        <is>
+          <t>4.7</t>
+        </is>
+      </c>
+      <c r="G75" s="2" t="inlineStr">
+        <is>
+          <t>E-commerce WhatsApp &amp; Turnos Peluquería</t>
+        </is>
+      </c>
+      <c r="H75" s="4" t="inlineStr">
+        <is>
+          <t>📲 Enviar Mensaje</t>
+        </is>
+      </c>
+      <c r="I75" s="5" t="inlineStr">
+        <is>
+          <t>🔗 Probar Boceto</t>
+        </is>
+      </c>
+      <c r="J75" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="K75" s="2" t="inlineStr"/>
+      <c r="L75" s="7" t="inlineStr">
+        <is>
+          <t>Ver en Maps</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="22" customHeight="1">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>GINEBRA PET SHOP</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>GINEBRA PET SHOP</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="inlineStr">
+        <is>
+          <t>Mascotas / Pet Shop</t>
+        </is>
+      </c>
+      <c r="D76" s="2" t="inlineStr">
+        <is>
+          <t>011 15-3080-4293</t>
+        </is>
+      </c>
+      <c r="E76" s="2" t="inlineStr">
+        <is>
+          <t>Chivilcoy 2590, C1417 Cdad. Autónoma de Buenos Aires</t>
+        </is>
+      </c>
+      <c r="F76" s="3" t="inlineStr">
+        <is>
+          <t>4.8</t>
+        </is>
+      </c>
+      <c r="G76" s="2" t="inlineStr">
+        <is>
+          <t>E-commerce WhatsApp &amp; Turnos Peluquería</t>
+        </is>
+      </c>
+      <c r="H76" s="4" t="inlineStr">
+        <is>
+          <t>📲 Enviar Mensaje</t>
+        </is>
+      </c>
+      <c r="I76" s="5" t="inlineStr">
+        <is>
+          <t>🔗 Probar Boceto</t>
+        </is>
+      </c>
+      <c r="J76" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="K76" s="2" t="inlineStr"/>
+      <c r="L76" s="7" t="inlineStr">
+        <is>
+          <t>Ver en Maps</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="22" customHeight="1">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>Lucky Pets</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>Lucky Pets</t>
+        </is>
+      </c>
+      <c r="C77" s="2" t="inlineStr">
+        <is>
+          <t>Mascotas / Pet Shop</t>
+        </is>
+      </c>
+      <c r="D77" s="2" t="inlineStr">
+        <is>
+          <t>011 7064-2536</t>
+        </is>
+      </c>
+      <c r="E77" s="2" t="inlineStr">
+        <is>
+          <t>Av. Francisco Beiró 5047, C1419HZM Cdad. Autónoma de Buenos Aires</t>
+        </is>
+      </c>
+      <c r="F77" s="3" t="inlineStr">
+        <is>
+          <t>4.9</t>
+        </is>
+      </c>
+      <c r="G77" s="2" t="inlineStr">
+        <is>
+          <t>E-commerce WhatsApp &amp; Turnos Peluquería</t>
+        </is>
+      </c>
+      <c r="H77" s="4" t="inlineStr">
+        <is>
+          <t>📲 Enviar Mensaje</t>
+        </is>
+      </c>
+      <c r="I77" s="5" t="inlineStr">
+        <is>
+          <t>🔗 Probar Boceto</t>
+        </is>
+      </c>
+      <c r="J77" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="K77" s="2" t="inlineStr"/>
+      <c r="L77" s="7" t="inlineStr">
+        <is>
+          <t>Ver en Maps</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="22" customHeight="1">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>Sky Vet Pet Shop y Clínica Veterinaria</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>Sky Vet Pet Shop y Clínica Veterinaria</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>Mascotas / Pet Shop</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="inlineStr">
+        <is>
+          <t>011 3135-4597</t>
+        </is>
+      </c>
+      <c r="E78" s="2" t="inlineStr">
+        <is>
+          <t>C. Llavallol 4393, C1419 Cdad. Autónoma de Buenos Aires</t>
+        </is>
+      </c>
+      <c r="F78" s="3" t="inlineStr">
+        <is>
+          <t>4.9</t>
+        </is>
+      </c>
+      <c r="G78" s="2" t="inlineStr">
+        <is>
+          <t>E-commerce WhatsApp &amp; Turnos Peluquería</t>
+        </is>
+      </c>
+      <c r="H78" s="4" t="inlineStr">
+        <is>
+          <t>📲 Enviar Mensaje</t>
+        </is>
+      </c>
+      <c r="I78" s="5" t="inlineStr">
+        <is>
+          <t>🔗 Probar Boceto</t>
+        </is>
+      </c>
+      <c r="J78" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="K78" s="2" t="inlineStr"/>
+      <c r="L78" s="7" t="inlineStr">
+        <is>
+          <t>Ver en Maps</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="22" customHeight="1">
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>Pet Shop Bros Hermanos Risso</t>
+        </is>
+      </c>
+      <c r="B79" s="2" t="inlineStr">
+        <is>
+          <t>Pet Shop Bros Hermanos Risso</t>
+        </is>
+      </c>
+      <c r="C79" s="2" t="inlineStr">
+        <is>
+          <t>Mascotas / Pet Shop</t>
+        </is>
+      </c>
+      <c r="D79" s="2" t="inlineStr">
+        <is>
+          <t>011 6002-5050</t>
+        </is>
+      </c>
+      <c r="E79" s="2" t="inlineStr">
+        <is>
+          <t>Nogoyá 3688, C1417 Cdad. Autónoma de Buenos Aires</t>
+        </is>
+      </c>
+      <c r="F79" s="3" t="inlineStr">
+        <is>
+          <t>4.9</t>
+        </is>
+      </c>
+      <c r="G79" s="2" t="inlineStr">
+        <is>
+          <t>E-commerce WhatsApp &amp; Turnos Peluquería</t>
+        </is>
+      </c>
+      <c r="H79" s="4" t="inlineStr">
+        <is>
+          <t>📲 Enviar Mensaje</t>
+        </is>
+      </c>
+      <c r="I79" s="5" t="inlineStr">
+        <is>
+          <t>🔗 Probar Boceto</t>
+        </is>
+      </c>
+      <c r="J79" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="K79" s="2" t="inlineStr"/>
+      <c r="L79" s="7" t="inlineStr">
+        <is>
+          <t>Ver en Maps</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" ht="22" customHeight="1">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>Pet shop Peluquería Canina "Don Fleco"</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>Pet shop Peluquería Canina Don Fleco</t>
+        </is>
+      </c>
+      <c r="C80" s="2" t="inlineStr">
+        <is>
+          <t>Mascotas / Pet Shop</t>
+        </is>
+      </c>
+      <c r="D80" s="2" t="inlineStr">
+        <is>
+          <t>011 2480-2127</t>
+        </is>
+      </c>
+      <c r="E80" s="2" t="inlineStr">
+        <is>
+          <t>Olleros 4145, C1427 EEM, Cdad. Autónoma de Buenos Aires</t>
+        </is>
+      </c>
+      <c r="F80" s="3" t="inlineStr">
+        <is>
+          <t>4.5</t>
+        </is>
+      </c>
+      <c r="G80" s="2" t="inlineStr">
+        <is>
+          <t>E-commerce WhatsApp &amp; Turnos Peluquería</t>
+        </is>
+      </c>
+      <c r="H80" s="4" t="inlineStr">
+        <is>
+          <t>📲 Enviar Mensaje</t>
+        </is>
+      </c>
+      <c r="I80" s="5" t="inlineStr">
+        <is>
+          <t>🔗 Probar Boceto</t>
+        </is>
+      </c>
+      <c r="J80" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="K80" s="2" t="inlineStr"/>
+      <c r="L80" s="7" t="inlineStr">
+        <is>
+          <t>Ver en Maps</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" ht="22" customHeight="1">
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>Del Carril Pet Shop Colegiales</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>Del Carril Pet Shop Colegiales</t>
+        </is>
+      </c>
+      <c r="C81" s="2" t="inlineStr">
+        <is>
+          <t>Mascotas / Pet Shop</t>
+        </is>
+      </c>
+      <c r="D81" s="2" t="inlineStr">
+        <is>
+          <t>011 7148-2124</t>
+        </is>
+      </c>
+      <c r="E81" s="2" t="inlineStr">
+        <is>
+          <t>Av. Elcano 3088, C1428 Cdad. Autónoma de Buenos Aires</t>
+        </is>
+      </c>
+      <c r="F81" s="3" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="G81" s="2" t="inlineStr">
+        <is>
+          <t>E-commerce WhatsApp &amp; Turnos Peluquería</t>
+        </is>
+      </c>
+      <c r="H81" s="4" t="inlineStr">
+        <is>
+          <t>📲 Enviar Mensaje</t>
+        </is>
+      </c>
+      <c r="I81" s="5" t="inlineStr">
+        <is>
+          <t>🔗 Probar Boceto</t>
+        </is>
+      </c>
+      <c r="J81" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="K81" s="2" t="inlineStr"/>
+      <c r="L81" s="7" t="inlineStr">
+        <is>
+          <t>Ver en Maps</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="22" customHeight="1">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>Pet Shop Huellas de Luz</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>Pet Shop Huellas de Luz</t>
+        </is>
+      </c>
+      <c r="C82" s="2" t="inlineStr">
+        <is>
+          <t>Mascotas / Pet Shop</t>
+        </is>
+      </c>
+      <c r="D82" s="2" t="inlineStr">
+        <is>
+          <t>011 3006-9299</t>
+        </is>
+      </c>
+      <c r="E82" s="2" t="inlineStr">
+        <is>
+          <t>Av. Forest 409, C1427 Cdad. Autónoma de Buenos Aires</t>
+        </is>
+      </c>
+      <c r="F82" s="3" t="inlineStr">
+        <is>
+          <t>4.2</t>
+        </is>
+      </c>
+      <c r="G82" s="2" t="inlineStr">
+        <is>
+          <t>E-commerce WhatsApp &amp; Turnos Peluquería</t>
+        </is>
+      </c>
+      <c r="H82" s="4" t="inlineStr">
+        <is>
+          <t>📲 Enviar Mensaje</t>
+        </is>
+      </c>
+      <c r="I82" s="5" t="inlineStr">
+        <is>
+          <t>🔗 Probar Boceto</t>
+        </is>
+      </c>
+      <c r="J82" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="K82" s="2" t="inlineStr"/>
+      <c r="L82" s="7" t="inlineStr">
+        <is>
+          <t>Ver en Maps</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="22" customHeight="1">
+      <c r="A83" s="2" t="inlineStr">
+        <is>
+          <t>Piccoli Pet</t>
+        </is>
+      </c>
+      <c r="B83" s="2" t="inlineStr">
+        <is>
+          <t>Piccoli Pet</t>
+        </is>
+      </c>
+      <c r="C83" s="2" t="inlineStr">
+        <is>
+          <t>Mascotas / Pet Shop</t>
+        </is>
+      </c>
+      <c r="D83" s="2" t="inlineStr">
+        <is>
+          <t>011 4765-6892</t>
+        </is>
+      </c>
+      <c r="E83" s="2" t="inlineStr">
+        <is>
+          <t>Dorrego 1541, C1414CKK Cdad. Autónoma de Buenos Aires</t>
+        </is>
+      </c>
+      <c r="F83" s="3" t="inlineStr">
+        <is>
+          <t>4.2</t>
+        </is>
+      </c>
+      <c r="G83" s="2" t="inlineStr">
+        <is>
+          <t>E-commerce WhatsApp &amp; Turnos Peluquería</t>
+        </is>
+      </c>
+      <c r="H83" s="4" t="inlineStr">
+        <is>
+          <t>📲 Enviar Mensaje</t>
+        </is>
+      </c>
+      <c r="I83" s="5" t="inlineStr">
+        <is>
+          <t>🔗 Probar Boceto</t>
+        </is>
+      </c>
+      <c r="J83" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="K83" s="2" t="inlineStr"/>
+      <c r="L83" s="7" t="inlineStr">
+        <is>
+          <t>Ver en Maps</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="22" customHeight="1">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>Menta Spa canino</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>Menta Spa canino</t>
+        </is>
+      </c>
+      <c r="C84" s="2" t="inlineStr">
+        <is>
+          <t>Mascotas / Pet Shop</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="inlineStr">
+        <is>
+          <t>011 6224-4416</t>
+        </is>
+      </c>
+      <c r="E84" s="2" t="inlineStr">
+        <is>
+          <t>Manzanares 4078, C1430AEN Cdad. Autónoma de Buenos Aires</t>
+        </is>
+      </c>
+      <c r="F84" s="3" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="G84" s="2" t="inlineStr">
+        <is>
+          <t>E-commerce WhatsApp &amp; Turnos Peluquería</t>
+        </is>
+      </c>
+      <c r="H84" s="4" t="inlineStr">
+        <is>
+          <t>📲 Enviar Mensaje</t>
+        </is>
+      </c>
+      <c r="I84" s="5" t="inlineStr">
+        <is>
+          <t>🔗 Probar Boceto</t>
+        </is>
+      </c>
+      <c r="J84" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="K84" s="2" t="inlineStr"/>
+      <c r="L84" s="7" t="inlineStr">
+        <is>
+          <t>Ver en Maps</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" ht="22" customHeight="1">
+      <c r="A85" s="2" t="inlineStr">
+        <is>
+          <t>COQUETES PET-SHOP</t>
+        </is>
+      </c>
+      <c r="B85" s="2" t="inlineStr">
+        <is>
+          <t>COQUETES PET-SHOP</t>
+        </is>
+      </c>
+      <c r="C85" s="2" t="inlineStr">
+        <is>
+          <t>Mascotas / Pet Shop</t>
+        </is>
+      </c>
+      <c r="D85" s="2" t="inlineStr">
+        <is>
+          <t>011 4546-0024</t>
+        </is>
+      </c>
+      <c r="E85" s="2" t="inlineStr">
+        <is>
+          <t>Crisólogo Larralde 3652, C1430 AIF, Cdad. Autónoma de Buenos Aires</t>
+        </is>
+      </c>
+      <c r="F85" s="3" t="inlineStr">
+        <is>
+          <t>4.8</t>
+        </is>
+      </c>
+      <c r="G85" s="2" t="inlineStr">
+        <is>
+          <t>E-commerce WhatsApp &amp; Turnos Peluquería</t>
+        </is>
+      </c>
+      <c r="H85" s="4" t="inlineStr">
+        <is>
+          <t>📲 Enviar Mensaje</t>
+        </is>
+      </c>
+      <c r="I85" s="5" t="inlineStr">
+        <is>
+          <t>🔗 Probar Boceto</t>
+        </is>
+      </c>
+      <c r="J85" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="K85" s="2" t="inlineStr"/>
+      <c r="L85" s="7" t="inlineStr">
+        <is>
+          <t>Ver en Maps</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="22" customHeight="1">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>Pet Shop Lumi</t>
+        </is>
+      </c>
+      <c r="B86" s="2" t="inlineStr">
+        <is>
+          <t>Pet Shop Lumi</t>
+        </is>
+      </c>
+      <c r="C86" s="2" t="inlineStr">
+        <is>
+          <t>Mascotas / Pet Shop</t>
+        </is>
+      </c>
+      <c r="D86" s="2" t="inlineStr">
+        <is>
+          <t>011 4704-9942</t>
+        </is>
+      </c>
+      <c r="E86" s="2" t="inlineStr">
+        <is>
+          <t>Av. García del Río 2487, C1429 DEA, Cdad. Autónoma de Buenos Aires</t>
+        </is>
+      </c>
+      <c r="F86" s="3" t="inlineStr">
+        <is>
+          <t>3.9</t>
+        </is>
+      </c>
+      <c r="G86" s="2" t="inlineStr">
+        <is>
+          <t>E-commerce WhatsApp &amp; Turnos Peluquería</t>
+        </is>
+      </c>
+      <c r="H86" s="4" t="inlineStr">
+        <is>
+          <t>📲 Enviar Mensaje</t>
+        </is>
+      </c>
+      <c r="I86" s="5" t="inlineStr">
+        <is>
+          <t>🔗 Probar Boceto</t>
+        </is>
+      </c>
+      <c r="J86" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="K86" s="2" t="inlineStr"/>
+      <c r="L86" s="7" t="inlineStr">
+        <is>
+          <t>Ver en Maps</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="22" customHeight="1">
+      <c r="A87" s="2" t="inlineStr">
+        <is>
+          <t>Peluqueria canina Pulguitas saavedra</t>
+        </is>
+      </c>
+      <c r="B87" s="2" t="inlineStr">
+        <is>
+          <t>Peluqueria canina Pulguitas saavedra</t>
+        </is>
+      </c>
+      <c r="C87" s="2" t="inlineStr">
+        <is>
+          <t>Mascotas / Pet Shop</t>
+        </is>
+      </c>
+      <c r="D87" s="2" t="inlineStr">
+        <is>
+          <t>011 5799-1340</t>
+        </is>
+      </c>
+      <c r="E87" s="2" t="inlineStr">
+        <is>
+          <t>Av. Ruiz Huidobro 3890, C1430 Cdad. Autónoma de Buenos Aires</t>
+        </is>
+      </c>
+      <c r="F87" s="3" t="inlineStr">
+        <is>
+          <t>4.0</t>
+        </is>
+      </c>
+      <c r="G87" s="2" t="inlineStr">
+        <is>
+          <t>E-commerce WhatsApp &amp; Turnos Peluquería</t>
+        </is>
+      </c>
+      <c r="H87" s="4" t="inlineStr">
+        <is>
+          <t>📲 Enviar Mensaje</t>
+        </is>
+      </c>
+      <c r="I87" s="5" t="inlineStr">
+        <is>
+          <t>🔗 Probar Boceto</t>
+        </is>
+      </c>
+      <c r="J87" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="K87" s="2" t="inlineStr"/>
+      <c r="L87" s="7" t="inlineStr">
+        <is>
+          <t>Ver en Maps</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" ht="22" customHeight="1">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>La Mascoteria</t>
+        </is>
+      </c>
+      <c r="B88" s="2" t="inlineStr">
+        <is>
+          <t>La Mascoteria</t>
+        </is>
+      </c>
+      <c r="C88" s="2" t="inlineStr">
+        <is>
+          <t>Mascotas / Pet Shop</t>
+        </is>
+      </c>
+      <c r="D88" s="2" t="inlineStr">
+        <is>
+          <t>011 5752-7066</t>
+        </is>
+      </c>
+      <c r="E88" s="2" t="inlineStr">
+        <is>
+          <t>Vuelta de Obligado 3217, C1429 Cdad. Autónoma de Buenos Aires</t>
+        </is>
+      </c>
+      <c r="F88" s="3" t="inlineStr">
+        <is>
+          <t>4.6</t>
+        </is>
+      </c>
+      <c r="G88" s="2" t="inlineStr">
+        <is>
+          <t>E-commerce WhatsApp &amp; Turnos Peluquería</t>
+        </is>
+      </c>
+      <c r="H88" s="4" t="inlineStr">
+        <is>
+          <t>📲 Enviar Mensaje</t>
+        </is>
+      </c>
+      <c r="I88" s="5" t="inlineStr">
+        <is>
+          <t>🔗 Probar Boceto</t>
+        </is>
+      </c>
+      <c r="J88" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="K88" s="2" t="inlineStr"/>
+      <c r="L88" s="7" t="inlineStr">
+        <is>
+          <t>Ver en Maps</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" ht="22" customHeight="1">
+      <c r="A89" s="2" t="inlineStr">
+        <is>
+          <t>Pet Shop Del Parque</t>
+        </is>
+      </c>
+      <c r="B89" s="2" t="inlineStr">
+        <is>
+          <t>Pet Shop Del Parque</t>
+        </is>
+      </c>
+      <c r="C89" s="2" t="inlineStr">
+        <is>
+          <t>Mascotas / Pet Shop</t>
+        </is>
+      </c>
+      <c r="D89" s="2" t="inlineStr">
+        <is>
+          <t>011 6528-8874</t>
+        </is>
+      </c>
+      <c r="E89" s="2" t="inlineStr">
+        <is>
+          <t>Conde 3609, C1430FHO Cdad. Autónoma de Buenos Aires</t>
+        </is>
+      </c>
+      <c r="F89" s="3" t="inlineStr">
+        <is>
+          <t>4.6</t>
+        </is>
+      </c>
+      <c r="G89" s="2" t="inlineStr">
+        <is>
+          <t>E-commerce WhatsApp &amp; Turnos Peluquería</t>
+        </is>
+      </c>
+      <c r="H89" s="4" t="inlineStr">
+        <is>
+          <t>📲 Enviar Mensaje</t>
+        </is>
+      </c>
+      <c r="I89" s="5" t="inlineStr">
+        <is>
+          <t>🔗 Probar Boceto</t>
+        </is>
+      </c>
+      <c r="J89" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="K89" s="2" t="inlineStr"/>
+      <c r="L89" s="7" t="inlineStr">
+        <is>
+          <t>Ver en Maps</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" ht="22" customHeight="1">
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>Pet Shop La Tata</t>
+        </is>
+      </c>
+      <c r="B90" s="2" t="inlineStr">
+        <is>
+          <t>Pet Shop La Tata</t>
+        </is>
+      </c>
+      <c r="C90" s="2" t="inlineStr">
+        <is>
+          <t>Mascotas / Pet Shop</t>
+        </is>
+      </c>
+      <c r="D90" s="2" t="inlineStr">
+        <is>
+          <t>011 3006-2509</t>
+        </is>
+      </c>
+      <c r="E90" s="2" t="inlineStr">
+        <is>
+          <t>Crisólogo Larralde 4699, C1430 Cdad. Autónoma de Buenos Aires</t>
+        </is>
+      </c>
+      <c r="F90" s="3" t="inlineStr">
+        <is>
+          <t>4.5</t>
+        </is>
+      </c>
+      <c r="G90" s="2" t="inlineStr">
+        <is>
+          <t>E-commerce WhatsApp &amp; Turnos Peluquería</t>
+        </is>
+      </c>
+      <c r="H90" s="4" t="inlineStr">
+        <is>
+          <t>📲 Enviar Mensaje</t>
+        </is>
+      </c>
+      <c r="I90" s="5" t="inlineStr">
+        <is>
+          <t>🔗 Probar Boceto</t>
+        </is>
+      </c>
+      <c r="J90" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="K90" s="2" t="inlineStr"/>
+      <c r="L90" s="7" t="inlineStr">
+        <is>
+          <t>Ver en Maps</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" ht="22" customHeight="1">
+      <c r="A91" s="2" t="inlineStr">
+        <is>
+          <t>Adrian Peluqueria Canina y Pet Shop</t>
+        </is>
+      </c>
+      <c r="B91" s="2" t="inlineStr">
+        <is>
+          <t>Adrian Peluqueria Canina y Pet Shop</t>
+        </is>
+      </c>
+      <c r="C91" s="2" t="inlineStr">
+        <is>
+          <t>Mascotas / Pet Shop</t>
+        </is>
+      </c>
+      <c r="D91" s="2" t="inlineStr">
+        <is>
+          <t>011 5967-7343</t>
+        </is>
+      </c>
+      <c r="E91" s="2" t="inlineStr">
+        <is>
+          <t>Roque Pérez 2753, C1430FBE C1430FBE C1430FBE, Cdad. Autónoma de Buenos Aires</t>
+        </is>
+      </c>
+      <c r="F91" s="3" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="G91" s="2" t="inlineStr">
+        <is>
+          <t>E-commerce WhatsApp &amp; Turnos Peluquería</t>
+        </is>
+      </c>
+      <c r="H91" s="4" t="inlineStr">
+        <is>
+          <t>📲 Enviar Mensaje</t>
+        </is>
+      </c>
+      <c r="I91" s="5" t="inlineStr">
+        <is>
+          <t>🔗 Probar Boceto</t>
+        </is>
+      </c>
+      <c r="J91" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="K91" s="2" t="inlineStr"/>
+      <c r="L91" s="7" t="inlineStr">
+        <is>
+          <t>Ver en Maps</t>
+        </is>
+      </c>
+    </row>
+    <row r="92" ht="22" customHeight="1">
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t>Pet Shop Huesitos</t>
+        </is>
+      </c>
+      <c r="B92" s="2" t="inlineStr">
+        <is>
+          <t>Pet Shop Huesitos</t>
+        </is>
+      </c>
+      <c r="C92" s="2" t="inlineStr">
+        <is>
+          <t>Mascotas / Pet Shop</t>
+        </is>
+      </c>
+      <c r="D92" s="2" t="inlineStr">
+        <is>
+          <t>011 4867-6060</t>
+        </is>
+      </c>
+      <c r="E92" s="2" t="inlineStr">
+        <is>
+          <t>Av. Rivadavia 3207, C1203 AAE, Cdad. Autónoma de Buenos Aires</t>
+        </is>
+      </c>
+      <c r="F92" s="3" t="inlineStr">
+        <is>
+          <t>4.4</t>
+        </is>
+      </c>
+      <c r="G92" s="2" t="inlineStr">
+        <is>
+          <t>E-commerce WhatsApp &amp; Turnos Peluquería</t>
+        </is>
+      </c>
+      <c r="H92" s="4" t="inlineStr">
+        <is>
+          <t>📲 Enviar Mensaje</t>
+        </is>
+      </c>
+      <c r="I92" s="5" t="inlineStr">
+        <is>
+          <t>🔗 Probar Boceto</t>
+        </is>
+      </c>
+      <c r="J92" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="K92" s="2" t="inlineStr"/>
+      <c r="L92" s="7" t="inlineStr">
+        <is>
+          <t>Ver en Maps</t>
+        </is>
+      </c>
+    </row>
+    <row r="93" ht="22" customHeight="1">
+      <c r="A93" s="2" t="inlineStr">
+        <is>
+          <t>Veterinaria y Pet Shop "Los Canarios de Balvanera" - Asociación Argentina de Canaricultura Roller</t>
+        </is>
+      </c>
+      <c r="B93" s="2" t="inlineStr">
+        <is>
+          <t>Veterinaria y Pet Shop Los Canarios de Balvanera - Asociación Argentina de Canaricultura Roller</t>
+        </is>
+      </c>
+      <c r="C93" s="2" t="inlineStr">
+        <is>
+          <t>Mascotas / Pet Shop</t>
+        </is>
+      </c>
+      <c r="D93" s="2" t="inlineStr">
+        <is>
+          <t>011 2147-7696</t>
+        </is>
+      </c>
+      <c r="E93" s="2" t="inlineStr">
+        <is>
+          <t>Av. Rivadavia 2317, C1034ACC Cdad. Autónoma de Buenos Aires</t>
+        </is>
+      </c>
+      <c r="F93" s="3" t="inlineStr">
+        <is>
+          <t>4.4</t>
+        </is>
+      </c>
+      <c r="G93" s="2" t="inlineStr">
+        <is>
+          <t>E-commerce WhatsApp &amp; Turnos Peluquería</t>
+        </is>
+      </c>
+      <c r="H93" s="4" t="inlineStr">
+        <is>
+          <t>📲 Enviar Mensaje</t>
+        </is>
+      </c>
+      <c r="I93" s="5" t="inlineStr">
+        <is>
+          <t>🔗 Probar Boceto</t>
+        </is>
+      </c>
+      <c r="J93" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="K93" s="2" t="inlineStr"/>
+      <c r="L93" s="7" t="inlineStr">
+        <is>
+          <t>Ver en Maps</t>
+        </is>
+      </c>
+    </row>
+    <row r="94" ht="22" customHeight="1">
+      <c r="A94" s="2" t="inlineStr">
+        <is>
+          <t>Puppy Shop</t>
+        </is>
+      </c>
+      <c r="B94" s="2" t="inlineStr">
+        <is>
+          <t>Puppy Shop</t>
+        </is>
+      </c>
+      <c r="C94" s="2" t="inlineStr">
+        <is>
+          <t>Mascotas / Pet Shop</t>
+        </is>
+      </c>
+      <c r="D94" s="2" t="inlineStr">
+        <is>
+          <t>011 4373-2034</t>
+        </is>
+      </c>
+      <c r="E94" s="2" t="inlineStr">
+        <is>
+          <t>Moreno 1819, C1094 ABA, Cdad. Autónoma de Buenos Aires</t>
+        </is>
+      </c>
+      <c r="F94" s="3" t="inlineStr">
+        <is>
+          <t>4.0</t>
+        </is>
+      </c>
+      <c r="G94" s="2" t="inlineStr">
+        <is>
+          <t>E-commerce WhatsApp &amp; Turnos Peluquería</t>
+        </is>
+      </c>
+      <c r="H94" s="4" t="inlineStr">
+        <is>
+          <t>📲 Enviar Mensaje</t>
+        </is>
+      </c>
+      <c r="I94" s="5" t="inlineStr">
+        <is>
+          <t>🔗 Probar Boceto</t>
+        </is>
+      </c>
+      <c r="J94" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="K94" s="2" t="inlineStr"/>
+      <c r="L94" s="7" t="inlineStr">
+        <is>
+          <t>Ver en Maps</t>
+        </is>
+      </c>
+    </row>
+    <row r="95" ht="22" customHeight="1">
+      <c r="A95" s="2" t="inlineStr">
+        <is>
+          <t>Veterinaria Spinetto</t>
+        </is>
+      </c>
+      <c r="B95" s="2" t="inlineStr">
+        <is>
+          <t>Veterinaria Spinetto</t>
+        </is>
+      </c>
+      <c r="C95" s="2" t="inlineStr">
+        <is>
+          <t>Mascotas / Pet Shop</t>
+        </is>
+      </c>
+      <c r="D95" s="2" t="inlineStr">
+        <is>
+          <t>011 4952-5910</t>
+        </is>
+      </c>
+      <c r="E95" s="2" t="inlineStr">
+        <is>
+          <t>Moreno 2301, C1082 Cdad. Autónoma de Buenos Aires</t>
+        </is>
+      </c>
+      <c r="F95" s="3" t="inlineStr">
+        <is>
+          <t>3.9</t>
+        </is>
+      </c>
+      <c r="G95" s="2" t="inlineStr">
+        <is>
+          <t>E-commerce WhatsApp &amp; Turnos Peluquería</t>
+        </is>
+      </c>
+      <c r="H95" s="4" t="inlineStr">
+        <is>
+          <t>📲 Enviar Mensaje</t>
+        </is>
+      </c>
+      <c r="I95" s="5" t="inlineStr">
+        <is>
+          <t>🔗 Probar Boceto</t>
+        </is>
+      </c>
+      <c r="J95" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="K95" s="2" t="inlineStr"/>
+      <c r="L95" s="7" t="inlineStr">
+        <is>
+          <t>Ver en Maps</t>
+        </is>
+      </c>
+    </row>
+    <row r="96" ht="22" customHeight="1">
+      <c r="A96" s="2" t="inlineStr">
+        <is>
+          <t>Veterinaria del Centro</t>
+        </is>
+      </c>
+      <c r="B96" s="2" t="inlineStr">
+        <is>
+          <t>Veterinaria del Centro</t>
+        </is>
+      </c>
+      <c r="C96" s="2" t="inlineStr">
+        <is>
+          <t>Mascotas / Pet Shop</t>
+        </is>
+      </c>
+      <c r="D96" s="2" t="inlineStr">
+        <is>
+          <t>011 4954-0981</t>
+        </is>
+      </c>
+      <c r="E96" s="2" t="inlineStr">
+        <is>
+          <t>C. Pres. Jose E. Uriburu 662, C1027 AAN, Cdad. Autónoma de Buenos Aires</t>
+        </is>
+      </c>
+      <c r="F96" s="3" t="inlineStr">
+        <is>
+          <t>4.7</t>
+        </is>
+      </c>
+      <c r="G96" s="2" t="inlineStr">
+        <is>
+          <t>E-commerce WhatsApp &amp; Turnos Peluquería</t>
+        </is>
+      </c>
+      <c r="H96" s="4" t="inlineStr">
+        <is>
+          <t>📲 Enviar Mensaje</t>
+        </is>
+      </c>
+      <c r="I96" s="5" t="inlineStr">
+        <is>
+          <t>🔗 Probar Boceto</t>
+        </is>
+      </c>
+      <c r="J96" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="K96" s="2" t="inlineStr"/>
+      <c r="L96" s="7" t="inlineStr">
+        <is>
+          <t>Ver en Maps</t>
+        </is>
+      </c>
+    </row>
+    <row r="97" ht="22" customHeight="1">
+      <c r="A97" s="2" t="inlineStr">
+        <is>
+          <t>CLINICA VETERINARIA PLUTO</t>
+        </is>
+      </c>
+      <c r="B97" s="2" t="inlineStr">
+        <is>
+          <t>CLINICA VETERINARIA PLUTO</t>
+        </is>
+      </c>
+      <c r="C97" s="2" t="inlineStr">
+        <is>
+          <t>Mascotas / Pet Shop</t>
+        </is>
+      </c>
+      <c r="D97" s="2" t="inlineStr">
+        <is>
+          <t>011 4030-0979</t>
+        </is>
+      </c>
+      <c r="E97" s="2" t="inlineStr">
+        <is>
+          <t>La Rioja 488, C1214 Cdad. Autónoma de Buenos Aires</t>
+        </is>
+      </c>
+      <c r="F97" s="3" t="inlineStr">
+        <is>
+          <t>4.7</t>
+        </is>
+      </c>
+      <c r="G97" s="2" t="inlineStr">
+        <is>
+          <t>E-commerce WhatsApp &amp; Turnos Peluquería</t>
+        </is>
+      </c>
+      <c r="H97" s="4" t="inlineStr">
+        <is>
+          <t>📲 Enviar Mensaje</t>
+        </is>
+      </c>
+      <c r="I97" s="5" t="inlineStr">
+        <is>
+          <t>🔗 Probar Boceto</t>
+        </is>
+      </c>
+      <c r="J97" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="K97" s="2" t="inlineStr"/>
+      <c r="L97" s="7" t="inlineStr">
+        <is>
+          <t>Ver en Maps</t>
+        </is>
+      </c>
+    </row>
+    <row r="98" ht="22" customHeight="1">
+      <c r="A98" s="2" t="inlineStr">
+        <is>
+          <t>Pet shop y baño canino/ Free Pet</t>
+        </is>
+      </c>
+      <c r="B98" s="2" t="inlineStr">
+        <is>
+          <t>Pet shop y baño canino/ Free Pet</t>
+        </is>
+      </c>
+      <c r="C98" s="2" t="inlineStr">
+        <is>
+          <t>Mascotas / Pet Shop</t>
+        </is>
+      </c>
+      <c r="D98" s="2" t="inlineStr">
+        <is>
+          <t>011 7081-8915</t>
+        </is>
+      </c>
+      <c r="E98" s="2" t="inlineStr">
+        <is>
+          <t>Comuna 11, Av. Nazca 3271, C1417CVC Cdad. Autónoma de Buenos Aires</t>
+        </is>
+      </c>
+      <c r="F98" s="3" t="inlineStr">
+        <is>
+          <t>4.8</t>
+        </is>
+      </c>
+      <c r="G98" s="2" t="inlineStr">
+        <is>
+          <t>E-commerce WhatsApp &amp; Turnos Peluquería</t>
+        </is>
+      </c>
+      <c r="H98" s="4" t="inlineStr">
+        <is>
+          <t>📲 Enviar Mensaje</t>
+        </is>
+      </c>
+      <c r="I98" s="5" t="inlineStr">
+        <is>
+          <t>🔗 Probar Boceto</t>
+        </is>
+      </c>
+      <c r="J98" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="K98" s="2" t="inlineStr"/>
+      <c r="L98" s="7" t="inlineStr">
+        <is>
+          <t>Ver en Maps</t>
+        </is>
+      </c>
+    </row>
+    <row r="99" ht="22" customHeight="1">
+      <c r="A99" s="2" t="inlineStr">
+        <is>
+          <t>Zona Mascotas</t>
+        </is>
+      </c>
+      <c r="B99" s="2" t="inlineStr">
+        <is>
+          <t>Zona Mascotas</t>
+        </is>
+      </c>
+      <c r="C99" s="2" t="inlineStr">
+        <is>
+          <t>Mascotas / Pet Shop</t>
+        </is>
+      </c>
+      <c r="D99" s="2" t="inlineStr">
+        <is>
+          <t>011 2805-1496</t>
+        </is>
+      </c>
+      <c r="E99" s="2" t="inlineStr">
+        <is>
+          <t>Tinogasta 3289, C1417 Cdad. Autónoma de Buenos Aires</t>
+        </is>
+      </c>
+      <c r="F99" s="3" t="inlineStr">
+        <is>
+          <t>4.8</t>
+        </is>
+      </c>
+      <c r="G99" s="2" t="inlineStr">
+        <is>
+          <t>E-commerce WhatsApp &amp; Turnos Peluquería</t>
+        </is>
+      </c>
+      <c r="H99" s="4" t="inlineStr">
+        <is>
+          <t>📲 Enviar Mensaje</t>
+        </is>
+      </c>
+      <c r="I99" s="5" t="inlineStr">
+        <is>
+          <t>🔗 Probar Boceto</t>
+        </is>
+      </c>
+      <c r="J99" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="K99" s="2" t="inlineStr"/>
+      <c r="L99" s="7" t="inlineStr">
+        <is>
+          <t>Ver en Maps</t>
+        </is>
+      </c>
+    </row>
+    <row r="100" ht="22" customHeight="1">
+      <c r="A100" s="2" t="inlineStr">
+        <is>
+          <t>Pet's Club. "El club de las Mascotas"</t>
+        </is>
+      </c>
+      <c r="B100" s="2" t="inlineStr">
+        <is>
+          <t>Pets Club. El club de las Mascotas</t>
+        </is>
+      </c>
+      <c r="C100" s="2" t="inlineStr">
+        <is>
+          <t>Mascotas / Pet Shop</t>
+        </is>
+      </c>
+      <c r="D100" s="2" t="inlineStr">
+        <is>
+          <t>4828-2674</t>
+        </is>
+      </c>
+      <c r="E100" s="2" t="inlineStr">
+        <is>
+          <t>C1417AAG, Cuenca 2550, C1417 AAH, Cdad. Autónoma de Buenos Aires</t>
+        </is>
+      </c>
+      <c r="F100" s="3" t="inlineStr">
+        <is>
+          <t>4.5</t>
+        </is>
+      </c>
+      <c r="G100" s="2" t="inlineStr">
+        <is>
+          <t>E-commerce WhatsApp &amp; Turnos Peluquería</t>
+        </is>
+      </c>
+      <c r="H100" s="4" t="inlineStr">
+        <is>
+          <t>📲 Enviar Mensaje</t>
+        </is>
+      </c>
+      <c r="I100" s="5" t="inlineStr">
+        <is>
+          <t>🔗 Probar Boceto</t>
+        </is>
+      </c>
+      <c r="J100" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="K100" s="2" t="inlineStr"/>
+      <c r="L100" s="7" t="inlineStr">
+        <is>
+          <t>Ver en Maps</t>
+        </is>
+      </c>
+    </row>
+    <row r="101" ht="22" customHeight="1">
+      <c r="A101" s="2" t="inlineStr">
+        <is>
+          <t>PETSHOP JACUZZICAN</t>
+        </is>
+      </c>
+      <c r="B101" s="2" t="inlineStr">
+        <is>
+          <t>PETSHOP JACUZZICAN</t>
+        </is>
+      </c>
+      <c r="C101" s="2" t="inlineStr">
+        <is>
+          <t>Mascotas / Pet Shop</t>
+        </is>
+      </c>
+      <c r="D101" s="2" t="inlineStr">
+        <is>
+          <t>011 5045-1451</t>
+        </is>
+      </c>
+      <c r="E101" s="2" t="inlineStr">
+        <is>
+          <t>Nogoyá 3579, C1417FNO Cdad. Autónoma de Buenos Aires</t>
+        </is>
+      </c>
+      <c r="F101" s="3" t="inlineStr">
+        <is>
+          <t>4.9</t>
+        </is>
+      </c>
+      <c r="G101" s="2" t="inlineStr">
+        <is>
+          <t>E-commerce WhatsApp &amp; Turnos Peluquería</t>
+        </is>
+      </c>
+      <c r="H101" s="4" t="inlineStr">
+        <is>
+          <t>📲 Enviar Mensaje</t>
+        </is>
+      </c>
+      <c r="I101" s="5" t="inlineStr">
+        <is>
+          <t>🔗 Probar Boceto</t>
+        </is>
+      </c>
+      <c r="J101" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="K101" s="2" t="inlineStr"/>
+      <c r="L101" s="7" t="inlineStr">
+        <is>
+          <t>Ver en Maps</t>
+        </is>
+      </c>
+    </row>
+    <row r="102" ht="22" customHeight="1">
+      <c r="A102" s="2" t="inlineStr">
+        <is>
+          <t>PET'S FOOD</t>
+        </is>
+      </c>
+      <c r="B102" s="2" t="inlineStr">
+        <is>
+          <t>PETS FOOD</t>
+        </is>
+      </c>
+      <c r="C102" s="2" t="inlineStr">
+        <is>
+          <t>Mascotas / Pet Shop</t>
+        </is>
+      </c>
+      <c r="D102" s="2" t="inlineStr">
+        <is>
+          <t>011 4588-1951</t>
+        </is>
+      </c>
+      <c r="E102" s="2" t="inlineStr">
+        <is>
+          <t>Álvarez Jonte 2401, C1416EXJ Cdad. Autónoma de Buenos Aires</t>
+        </is>
+      </c>
+      <c r="F102" s="3" t="inlineStr">
+        <is>
+          <t>4.8</t>
+        </is>
+      </c>
+      <c r="G102" s="2" t="inlineStr">
+        <is>
+          <t>E-commerce WhatsApp &amp; Turnos Peluquería</t>
+        </is>
+      </c>
+      <c r="H102" s="4" t="inlineStr">
+        <is>
+          <t>📲 Enviar Mensaje</t>
+        </is>
+      </c>
+      <c r="I102" s="5" t="inlineStr">
+        <is>
+          <t>🔗 Probar Boceto</t>
+        </is>
+      </c>
+      <c r="J102" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="K102" s="2" t="inlineStr"/>
+      <c r="L102" s="7" t="inlineStr">
+        <is>
+          <t>Ver en Maps</t>
+        </is>
+      </c>
+    </row>
+    <row r="103" ht="22" customHeight="1">
+      <c r="A103" s="2" t="inlineStr">
+        <is>
+          <t>Acuario Willy's Pet Shop</t>
+        </is>
+      </c>
+      <c r="B103" s="2" t="inlineStr">
+        <is>
+          <t>Acuario Willys Pet Shop</t>
+        </is>
+      </c>
+      <c r="C103" s="2" t="inlineStr">
+        <is>
+          <t>Mascotas / Pet Shop</t>
+        </is>
+      </c>
+      <c r="D103" s="2" t="inlineStr">
+        <is>
+          <t>011 2403-9338</t>
+        </is>
+      </c>
+      <c r="E103" s="2" t="inlineStr">
+        <is>
+          <t>Nogoyá 3397, C1417FNK Cdad. Autónoma de Buenos Aires</t>
+        </is>
+      </c>
+      <c r="F103" s="3" t="inlineStr">
+        <is>
+          <t>4.6</t>
+        </is>
+      </c>
+      <c r="G103" s="2" t="inlineStr">
+        <is>
+          <t>E-commerce WhatsApp &amp; Turnos Peluquería</t>
+        </is>
+      </c>
+      <c r="H103" s="4" t="inlineStr">
+        <is>
+          <t>📲 Enviar Mensaje</t>
+        </is>
+      </c>
+      <c r="I103" s="5" t="inlineStr">
+        <is>
+          <t>🔗 Probar Boceto</t>
+        </is>
+      </c>
+      <c r="J103" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="K103" s="2" t="inlineStr"/>
+      <c r="L103" s="7" t="inlineStr">
+        <is>
+          <t>Ver en Maps</t>
+        </is>
+      </c>
+    </row>
+    <row r="104" ht="22" customHeight="1">
+      <c r="A104" s="2" t="inlineStr">
+        <is>
+          <t>Pet Shop Frodo</t>
+        </is>
+      </c>
+      <c r="B104" s="2" t="inlineStr">
+        <is>
+          <t>Pet Shop Frodo</t>
+        </is>
+      </c>
+      <c r="C104" s="2" t="inlineStr">
+        <is>
+          <t>Mascotas / Pet Shop</t>
+        </is>
+      </c>
+      <c r="D104" s="2" t="inlineStr">
+        <is>
+          <t>4504-1996</t>
+        </is>
+      </c>
+      <c r="E104" s="2" t="inlineStr">
+        <is>
+          <t>Baigorria 2320, C1417FQA C1417FQA, Cdad. Autónoma de Buenos Aires</t>
+        </is>
+      </c>
+      <c r="F104" s="3" t="inlineStr">
+        <is>
+          <t>4.1</t>
+        </is>
+      </c>
+      <c r="G104" s="2" t="inlineStr">
+        <is>
+          <t>E-commerce WhatsApp &amp; Turnos Peluquería</t>
+        </is>
+      </c>
+      <c r="H104" s="4" t="inlineStr">
+        <is>
+          <t>📲 Enviar Mensaje</t>
+        </is>
+      </c>
+      <c r="I104" s="5" t="inlineStr">
+        <is>
+          <t>🔗 Probar Boceto</t>
+        </is>
+      </c>
+      <c r="J104" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="K104" s="2" t="inlineStr"/>
+      <c r="L104" s="7" t="inlineStr">
+        <is>
+          <t>Ver en Maps</t>
+        </is>
+      </c>
+    </row>
+    <row r="105" ht="22" customHeight="1">
+      <c r="A105" s="2" t="inlineStr">
+        <is>
+          <t>Pupipet</t>
+        </is>
+      </c>
+      <c r="B105" s="2" t="inlineStr">
+        <is>
+          <t>Pupipet</t>
+        </is>
+      </c>
+      <c r="C105" s="2" t="inlineStr">
+        <is>
+          <t>Mascotas / Pet Shop</t>
+        </is>
+      </c>
+      <c r="D105" s="2" t="inlineStr">
+        <is>
+          <t>011 5370-3822</t>
+        </is>
+      </c>
+      <c r="E105" s="2" t="inlineStr">
+        <is>
+          <t>Emilio Lamarca 2036, C1407DGP Cdad. Autónoma de Buenos Aires</t>
+        </is>
+      </c>
+      <c r="F105" s="3" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="G105" s="2" t="inlineStr">
+        <is>
+          <t>E-commerce WhatsApp &amp; Turnos Peluquería</t>
+        </is>
+      </c>
+      <c r="H105" s="4" t="inlineStr">
+        <is>
+          <t>📲 Enviar Mensaje</t>
+        </is>
+      </c>
+      <c r="I105" s="5" t="inlineStr">
+        <is>
+          <t>🔗 Probar Boceto</t>
+        </is>
+      </c>
+      <c r="J105" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="K105" s="2" t="inlineStr"/>
+      <c r="L105" s="7" t="inlineStr">
+        <is>
+          <t>Ver en Maps</t>
+        </is>
+      </c>
+    </row>
+    <row r="106" ht="22" customHeight="1">
+      <c r="A106" s="2" t="inlineStr">
+        <is>
+          <t>Lo de Diógenes</t>
+        </is>
+      </c>
+      <c r="B106" s="2" t="inlineStr">
+        <is>
+          <t>Lo de Diógenes</t>
+        </is>
+      </c>
+      <c r="C106" s="2" t="inlineStr">
+        <is>
+          <t>Mascotas / Pet Shop</t>
+        </is>
+      </c>
+      <c r="D106" s="2" t="inlineStr">
+        <is>
+          <t>011 2302-0260</t>
+        </is>
+      </c>
+      <c r="E106" s="2" t="inlineStr">
+        <is>
+          <t>Cuenca 2695, C1417 Cdad. Autónoma de Buenos Aires</t>
+        </is>
+      </c>
+      <c r="F106" s="3" t="inlineStr">
+        <is>
+          <t>4.5</t>
+        </is>
+      </c>
+      <c r="G106" s="2" t="inlineStr">
+        <is>
+          <t>E-commerce WhatsApp &amp; Turnos Peluquería</t>
+        </is>
+      </c>
+      <c r="H106" s="4" t="inlineStr">
+        <is>
+          <t>📲 Enviar Mensaje</t>
+        </is>
+      </c>
+      <c r="I106" s="5" t="inlineStr">
+        <is>
+          <t>🔗 Probar Boceto</t>
+        </is>
+      </c>
+      <c r="J106" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="K106" s="2" t="inlineStr"/>
+      <c r="L106" s="7" t="inlineStr">
         <is>
           <t>Ver en Maps</t>
         </is>
@@ -3377,6 +6799,183 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H47" r:id="rId136"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I47" r:id="rId137"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L47" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H48" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I48" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L48" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H49" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I49" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L49" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H50" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I50" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L50" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H51" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I51" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L51" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H52" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I52" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L52" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H53" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I53" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L53" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H54" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I54" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L54" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H55" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I55" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L55" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H56" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I56" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L56" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H57" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I57" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L57" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H58" r:id="rId169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I58" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L58" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H59" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I59" r:id="rId173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L59" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H60" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I60" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L60" r:id="rId177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H61" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I61" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L61" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H62" r:id="rId181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I62" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L62" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H63" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I63" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L63" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H64" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I64" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L64" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H65" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I65" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L65" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H66" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I66" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L66" r:id="rId195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H67" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I67" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L67" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H68" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I68" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L68" r:id="rId201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H69" r:id="rId202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I69" r:id="rId203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L69" r:id="rId204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H70" r:id="rId205"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I70" r:id="rId206"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L70" r:id="rId207"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H71" r:id="rId208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I71" r:id="rId209"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L71" r:id="rId210"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H72" r:id="rId211"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I72" r:id="rId212"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L72" r:id="rId213"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H73" r:id="rId214"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I73" r:id="rId215"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L73" r:id="rId216"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H74" r:id="rId217"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I74" r:id="rId218"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L74" r:id="rId219"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H75" r:id="rId220"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I75" r:id="rId221"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L75" r:id="rId222"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H76" r:id="rId223"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I76" r:id="rId224"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L76" r:id="rId225"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H77" r:id="rId226"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I77" r:id="rId227"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L77" r:id="rId228"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H78" r:id="rId229"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I78" r:id="rId230"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L78" r:id="rId231"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H79" r:id="rId232"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I79" r:id="rId233"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L79" r:id="rId234"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H80" r:id="rId235"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I80" r:id="rId236"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L80" r:id="rId237"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H81" r:id="rId238"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I81" r:id="rId239"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L81" r:id="rId240"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H82" r:id="rId241"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I82" r:id="rId242"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L82" r:id="rId243"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H83" r:id="rId244"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I83" r:id="rId245"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L83" r:id="rId246"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H84" r:id="rId247"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I84" r:id="rId248"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L84" r:id="rId249"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H85" r:id="rId250"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I85" r:id="rId251"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L85" r:id="rId252"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H86" r:id="rId253"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I86" r:id="rId254"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L86" r:id="rId255"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H87" r:id="rId256"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I87" r:id="rId257"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L87" r:id="rId258"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H88" r:id="rId259"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I88" r:id="rId260"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L88" r:id="rId261"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H89" r:id="rId262"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I89" r:id="rId263"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L89" r:id="rId264"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H90" r:id="rId265"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I90" r:id="rId266"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L90" r:id="rId267"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H91" r:id="rId268"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I91" r:id="rId269"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L91" r:id="rId270"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H92" r:id="rId271"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I92" r:id="rId272"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L92" r:id="rId273"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H93" r:id="rId274"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I93" r:id="rId275"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L93" r:id="rId276"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H94" r:id="rId277"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I94" r:id="rId278"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L94" r:id="rId279"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H95" r:id="rId280"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I95" r:id="rId281"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L95" r:id="rId282"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H96" r:id="rId283"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I96" r:id="rId284"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L96" r:id="rId285"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H97" r:id="rId286"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I97" r:id="rId287"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L97" r:id="rId288"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H98" r:id="rId289"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I98" r:id="rId290"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L98" r:id="rId291"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H99" r:id="rId292"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I99" r:id="rId293"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L99" r:id="rId294"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H100" r:id="rId295"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I100" r:id="rId296"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L100" r:id="rId297"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H101" r:id="rId298"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I101" r:id="rId299"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L101" r:id="rId300"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H102" r:id="rId301"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I102" r:id="rId302"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L102" r:id="rId303"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H103" r:id="rId304"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I103" r:id="rId305"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L103" r:id="rId306"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H104" r:id="rId307"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I104" r:id="rId308"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L104" r:id="rId309"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H105" r:id="rId310"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I105" r:id="rId311"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L105" r:id="rId312"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H106" r:id="rId313"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I106" r:id="rId314"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L106" r:id="rId315"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>